<commit_message>
Link all BNC4 Excel valuation fields to effective daily pool price
</commit_message>
<xml_diff>
--- a/excel/latest/FourMeme_4Stock_BNC4_控筹模型.xlsx
+++ b/excel/latest/FourMeme_4Stock_BNC4_控筹模型.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="控筹模型" sheetId="1" r:id="Rffe7e1a924f44acc"/>
-    <sheet name="控筹测算" sheetId="2" r:id="Rd15db576cb5b4c33"/>
-    <sheet name="内外盘曲线" sheetId="3" r:id="R5319507f9c6c4c5e"/>
-    <sheet name="洗筹明细" sheetId="4" r:id="R0e2c89e81b7e455c"/>
-    <sheet name="参数与来源" sheetId="5" r:id="R65d0f1aaffda4dd3"/>
+    <sheet name="控筹模型" sheetId="1" r:id="R328ec81a6e794482"/>
+    <sheet name="控筹测算" sheetId="2" r:id="Rf163ef75fd0e425f"/>
+    <sheet name="内外盘曲线" sheetId="3" r:id="Re18391e927804b34"/>
+    <sheet name="洗筹明细" sheetId="4" r:id="R7f65398af3cc4597"/>
+    <sheet name="参数与来源" sheetId="5" r:id="R2e9a4f2059594bd8"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -4225,7 +4225,7 @@
         <v>BNC4 / USDT 价格</v>
       </c>
       <c r="D19" s="84">
-        <f>IF('控筹模型'!L14="","",'控筹模型'!L14)</f>
+        <f>IF('参数与来源'!$N$19="","",'参数与来源'!$N$19)</f>
       </c>
       <c r="E19" s="81" t="str">
         <v>可选；留空不输出 USD</v>

</xml_diff>

<commit_message>
Add Flap MYX workbook
</commit_message>
<xml_diff>
--- a/excel/latest/FourMeme_4Stock_BNC4_控筹模型.xlsx
+++ b/excel/latest/FourMeme_4Stock_BNC4_控筹模型.xlsx
@@ -4551,7 +4551,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>https://api.coingecko.com/api/v3/simple/price?ids=tether,ethereum,binancecoin,solana,hyperliquid,aster-2&amp;vs_currencies=usd&amp;include_last_updated_at=true</t>
+          <t>https://api.coingecko.com/api/v3/simple/price?ids=tether,ethereum,binancecoin,solana,hyperliquid,aster-2,myx-finance&amp;vs_currencies=usd&amp;include_last_updated_at=true</t>
         </is>
       </c>
       <c r="E8" s="5"/>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="AF14" s="21" t="inlineStr">
         <is>
-          <t>https://api.coingecko.com/api/v3/simple/price?ids=tether,ethereum,binancecoin,solana,hyperliquid,aster-2&amp;vs_currencies=usd&amp;include_last_updated_at=true</t>
+          <t>https://api.coingecko.com/api/v3/simple/price?ids=tether,ethereum,binancecoin,solana,hyperliquid,aster-2,myx-finance&amp;vs_currencies=usd&amp;include_last_updated_at=true</t>
         </is>
       </c>
       <c r="AG14" s="21" t="inlineStr">

</xml_diff>